<commit_message>
preloader and bulk upload fix
</commit_message>
<xml_diff>
--- a/public/product-import-template.xlsx
+++ b/public/product-import-template.xlsx
@@ -398,18 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J3"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="21.83203125" customWidth="1"/>
-    <col min="9" max="9" width="19.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -437,10 +425,10 @@
         <v>Low Stock Threshold</v>
       </c>
       <c r="I1" t="str">
-        <v>Short Description</v>
+        <v>Description</v>
       </c>
       <c r="J1" t="str">
-        <v>Description</v>
+        <v>Product Highlights</v>
       </c>
     </row>
     <row r="2">
@@ -472,7 +460,7 @@
         <v>A short one-line summary shown on product listings.</v>
       </c>
       <c r="J2" t="str">
-        <v>The full product description shown on the product page.</v>
+        <v>The full product highlights shown on the product page.</v>
       </c>
     </row>
     <row r="3">

</xml_diff>